<commit_message>
Ajout de la partie Data Jalon 2.1
</commit_message>
<xml_diff>
--- a/Tableau_amorcage_sources.xlsx
+++ b/Tableau_amorcage_sources.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alnof\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etudiant\Documents\SAE 3.01\SAE-3.01-2026-2027\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CD3CBF4-B850-4E13-BD0C-42BD8FA11AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32BDDD4B-1FA1-4D10-BD06-5587CD498BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="21336" windowHeight="11376" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau d'amorçage" sheetId="1" r:id="rId1"/>
@@ -31,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="95">
   <si>
     <t>Culture</t>
   </si>
@@ -318,13 +321,16 @@
   </si>
   <si>
     <t>Méditerranéen ; besoin de froid hivernal ; emblématique de la « remontée vers le nord »</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.semae-pedagogie.org/sujet/implantation-et-developpement/ </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -413,11 +419,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -440,9 +447,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
+    <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -744,7 +755,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N11"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -762,7 +773,7 @@
     <col min="14" max="14" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="30" customHeight="1">
+    <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -806,7 +817,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="91.5">
+    <row r="2" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
@@ -850,7 +861,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="76.5">
+    <row r="3" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>22</v>
       </c>
@@ -894,7 +905,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="91.5">
+    <row r="4" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>30</v>
       </c>
@@ -907,7 +918,9 @@
       <c r="D4" s="5">
         <v>2200</v>
       </c>
-      <c r="E4" s="4"/>
+      <c r="E4" s="8" t="s">
+        <v>94</v>
+      </c>
       <c r="F4" s="5">
         <v>-5</v>
       </c>
@@ -936,7 +949,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="76.5">
+    <row r="5" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>36</v>
       </c>
@@ -980,7 +993,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="106.5">
+    <row r="6" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>45</v>
       </c>
@@ -1024,7 +1037,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="60.75">
+    <row r="7" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>53</v>
       </c>
@@ -1068,7 +1081,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="91.5">
+    <row r="8" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>59</v>
       </c>
@@ -1112,7 +1125,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="152.25">
+    <row r="9" spans="1:14" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>67</v>
       </c>
@@ -1156,7 +1169,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="106.5">
+    <row r="10" spans="1:14" ht="105" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>76</v>
       </c>
@@ -1200,7 +1213,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="91.5">
+    <row r="11" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>85</v>
       </c>
@@ -1302,6 +1315,7 @@
     <hyperlink ref="I11" r:id="rId56" xr:uid="{27C59620-DB9A-454B-AD5E-243D9DC3993D}"/>
     <hyperlink ref="M11" r:id="rId57" xr:uid="{7767C8D2-67FB-4E51-A1A1-795892EC7403}"/>
     <hyperlink ref="M8" r:id="rId58" xr:uid="{344A1ECA-4868-4035-AAFD-B63242065260}"/>
+    <hyperlink ref="E4" r:id="rId59" xr:uid="{70287141-7BB7-45A6-A898-2606583A191A}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>